<commit_message>
Cap nhat file phan cong cong viec
</commit_message>
<xml_diff>
--- a/Phân Công Công Việc.xlsx
+++ b/Phân Công Công Việc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Phuc\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LTM_Caro_Online\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F6D9A99-5760-4C6E-8506-58CA961FDAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA51A1D9-5440-48DA-8F32-9FA429EABB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50184BE9-43ED-4868-BC23-3C567488F38F}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>Ngô Trương Tín</t>
   </si>
   <si>
-    <t xml:space="preserve">Code UI  Form Bàn cờ Caro </t>
-  </si>
-  <si>
     <t>Lê Tấn Đạt</t>
   </si>
   <si>
@@ -122,13 +119,16 @@
     <t>Code Chức năng Khán giả &amp; Lưu Lịch sử</t>
   </si>
   <si>
-    <t>Code Xử lý rớt mạng &amp; Ghi Log Server</t>
-  </si>
-  <si>
-    <t>Code Tạo phòng đấu</t>
-  </si>
-  <si>
-    <t>Code Giao diện Quản trị Server và Kiểm Thử</t>
+    <t>Code UI  Form Bàn cờ Caro, xử lý 1 số logic bàn cờ</t>
+  </si>
+  <si>
+    <t>Code Xử lý rớt mạng &amp; Ghi Log Server , xử lý 1 số logic bàn cờ</t>
+  </si>
+  <si>
+    <t>Code Tạo phòng đấu , làm báo cáo word</t>
+  </si>
+  <si>
+    <t>Code Giao diện Quản trị Server và Kiểm Thử, làm báo cáo word</t>
   </si>
 </sst>
 </file>
@@ -208,9 +208,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -221,6 +218,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -561,134 +561,134 @@
     <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="56.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>1</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="4" t="s">
+      <c r="E5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>2</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>9</v>
+      <c r="E6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>3</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="C7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>4</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>26</v>
+      <c r="C8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>5</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="C9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>6</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="4" t="s">
+      <c r="D10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>